<commit_message>
fix: remplace location/locationQualifier par l'extension includedStructure
bodyStructure-eu-core (Parent depuis le passage à l'héritage HL7 EU) interdit
location et locationQualifier (max 0) et les remplace par l'extension
includedStructure. Pointe les bindings (FRCoreValueSetBodyStructureLocation en
extensible, jdv-modificateur-topographique-cisis en required) vers les
sous-extensions structure et qualifier.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> a4b669805b3bef82b48082ec610438a95b2f66c9
</commit_message>
<xml_diff>
--- a/nr-doc-core-body-structure/ig/StructureDefinition-fr-core-body-structure.xlsx
+++ b/nr-doc-core-body-structure/ig/StructureDefinition-fr-core-body-structure.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3364" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3366" uniqueCount="406">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-28T08:49:31+00:00</t>
+    <t>2026-07-28T09:03:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -517,6 +517,9 @@
     <t>structure</t>
   </si>
   <si>
+    <t>Localisation anatomique ou voie d'abord</t>
+  </si>
+  <si>
     <t>BodyStructure.extension:includedStructure.extension:structure.id</t>
   </si>
   <si>
@@ -563,7 +566,10 @@
     <t>Code that represents the included structure.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/body-site|4.0.1</t>
+    <t>extensible</t>
+  </si>
+  <si>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-body-structure-location|2.2.0</t>
   </si>
   <si>
     <t>Extension.value[x]</t>
@@ -1031,6 +1037,9 @@
     <t>qualifier</t>
   </si>
   <si>
+    <t>Modificateurs topographiques</t>
+  </si>
+  <si>
     <t>BodyStructure.extension:includedStructure.extension:qualifier.id</t>
   </si>
   <si>
@@ -1049,7 +1058,10 @@
     <t>Code that represents the included structure qualifier.</t>
   </si>
   <si>
-    <t>http://hl7.eu/fhir/base/ValueSet/siteQualifier-eu|2.0.0</t>
+    <t>required</t>
+  </si>
+  <si>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-modificateur-topographique-cisis|20260619134042</t>
   </si>
   <si>
     <t>BodyStructure.extension:includedStructure.url</t>
@@ -1157,16 +1169,19 @@
     <t>BodyStructure.location</t>
   </si>
   <si>
-    <t>Localisation anatomique ou voie d'abord</t>
+    <t>Body site</t>
   </si>
   <si>
     <t>The anatomical location or region of the specimen, lesion, or body structure.</t>
   </si>
   <si>
-    <t>extensible</t>
-  </si>
-  <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-body-structure-location|2.2.0</t>
+    <t>example</t>
+  </si>
+  <si>
+    <t>Codes describing anatomical locations. May include laterality.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/body-site|4.0.1</t>
   </si>
   <si>
     <t>.targetSiteCode</t>
@@ -1181,16 +1196,16 @@
     <t>BodyStructure.locationQualifier</t>
   </si>
   <si>
-    <t>Modificateurs topographiques</t>
+    <t>Body site modifier</t>
   </si>
   <si>
     <t>Qualifier to refine the anatomical location.  These include qualifiers for laterality, relative location, directionality, number, and plane.</t>
   </si>
   <si>
-    <t>required</t>
-  </si>
-  <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-modificateur-topographique-cisis|20260619134042</t>
+    <t>Concepts modifying the anatomic location.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/bodystructure-relative-location|4.0.1</t>
   </si>
   <si>
     <t>Combines Side, Numerical identifier, Anatomical plane,and Aspect</t>
@@ -1598,7 +1613,7 @@
     <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="18.49609375" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="49.63671875" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="76.125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
@@ -3014,7 +3029,7 @@
         <v>134</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>135</v>
+        <v>161</v>
       </c>
       <c r="M13" t="s" s="2">
         <v>136</v>
@@ -3097,10 +3112,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -3209,10 +3224,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -3321,10 +3336,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -3350,13 +3365,13 @@
         <v>103</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N16" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O16" s="2"/>
       <c r="P16" t="s" s="2">
@@ -3406,7 +3421,7 @@
         <v>81</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>89</v>
@@ -3435,10 +3450,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3461,13 +3476,13 @@
         <v>81</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -3494,11 +3509,11 @@
         <v>81</v>
       </c>
       <c r="X17" t="s" s="2">
-        <v>113</v>
+        <v>177</v>
       </c>
       <c r="Y17" s="2"/>
       <c r="Z17" t="s" s="2">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="AA17" t="s" s="2">
         <v>81</v>
@@ -3516,7 +3531,7 @@
         <v>81</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>79</v>
@@ -3545,13 +3560,13 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B18" t="s" s="2">
         <v>156</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D18" t="s" s="2">
         <v>81</v>
@@ -3659,10 +3674,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3771,10 +3786,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -3883,10 +3898,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3912,13 +3927,13 @@
         <v>103</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N21" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
@@ -3926,7 +3941,7 @@
       </c>
       <c r="Q21" s="2"/>
       <c r="R21" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="S21" t="s" s="2">
         <v>81</v>
@@ -3968,7 +3983,7 @@
         <v>81</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>89</v>
@@ -3997,10 +4012,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4023,13 +4038,13 @@
         <v>81</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -4060,7 +4075,7 @@
       </c>
       <c r="Y22" s="2"/>
       <c r="Z22" t="s" s="2">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>81</v>
@@ -4078,7 +4093,7 @@
         <v>81</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>79</v>
@@ -4107,13 +4122,13 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B23" t="s" s="2">
         <v>156</v>
       </c>
       <c r="C23" t="s" s="2">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D23" t="s" s="2">
         <v>81</v>
@@ -4138,16 +4153,16 @@
         <v>134</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="O23" t="s" s="2">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="P23" t="s" s="2">
         <v>81</v>
@@ -4225,10 +4240,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4337,10 +4352,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4449,13 +4464,13 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C26" t="s" s="2">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D26" t="s" s="2">
         <v>81</v>
@@ -4480,16 +4495,16 @@
         <v>134</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="O26" t="s" s="2">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>81</v>
@@ -4567,10 +4582,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4679,14 +4694,14 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
@@ -4708,13 +4723,13 @@
         <v>134</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -4793,10 +4808,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4822,13 +4837,13 @@
         <v>103</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
@@ -4836,7 +4851,7 @@
       </c>
       <c r="Q29" s="2"/>
       <c r="R29" t="s" s="2">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="S29" t="s" s="2">
         <v>81</v>
@@ -4878,7 +4893,7 @@
         <v>81</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>89</v>
@@ -4907,10 +4922,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4933,13 +4948,13 @@
         <v>81</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -4990,7 +5005,7 @@
         <v>81</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>79</v>
@@ -5019,13 +5034,13 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C31" t="s" s="2">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D31" t="s" s="2">
         <v>81</v>
@@ -5050,16 +5065,16 @@
         <v>134</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="O31" t="s" s="2">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="P31" t="s" s="2">
         <v>81</v>
@@ -5137,10 +5152,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5249,14 +5264,14 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
@@ -5278,13 +5293,13 @@
         <v>134</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -5363,10 +5378,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5392,13 +5407,13 @@
         <v>103</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
@@ -5406,7 +5421,7 @@
       </c>
       <c r="Q34" s="2"/>
       <c r="R34" t="s" s="2">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="S34" t="s" s="2">
         <v>81</v>
@@ -5448,7 +5463,7 @@
         <v>81</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>89</v>
@@ -5477,10 +5492,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5503,13 +5518,13 @@
         <v>81</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -5560,7 +5575,7 @@
         <v>81</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>79</v>
@@ -5589,13 +5604,13 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C36" t="s" s="2">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D36" t="s" s="2">
         <v>81</v>
@@ -5620,16 +5635,16 @@
         <v>134</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="O36" t="s" s="2">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>81</v>
@@ -5707,10 +5722,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5819,10 +5834,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5931,13 +5946,13 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C39" t="s" s="2">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D39" t="s" s="2">
         <v>81</v>
@@ -5962,16 +5977,16 @@
         <v>134</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="N39" t="s" s="2">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="O39" t="s" s="2">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="P39" t="s" s="2">
         <v>81</v>
@@ -6049,10 +6064,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6161,10 +6176,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6273,13 +6288,13 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C42" t="s" s="2">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D42" t="s" s="2">
         <v>81</v>
@@ -6304,10 +6319,10 @@
         <v>134</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6387,10 +6402,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6499,14 +6514,14 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -6528,13 +6543,13 @@
         <v>134</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="N44" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
@@ -6613,10 +6628,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6642,13 +6657,13 @@
         <v>103</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N45" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
@@ -6656,7 +6671,7 @@
       </c>
       <c r="Q45" s="2"/>
       <c r="R45" t="s" s="2">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="S45" t="s" s="2">
         <v>81</v>
@@ -6698,7 +6713,7 @@
         <v>81</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>89</v>
@@ -6727,10 +6742,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6756,13 +6771,13 @@
         <v>150</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6770,7 +6785,7 @@
       </c>
       <c r="Q46" s="2"/>
       <c r="R46" t="s" s="2">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="S46" t="s" s="2">
         <v>81</v>
@@ -6812,7 +6827,7 @@
         <v>81</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>79</v>
@@ -6841,13 +6856,13 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C47" t="s" s="2">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D47" t="s" s="2">
         <v>81</v>
@@ -6872,16 +6887,16 @@
         <v>134</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="O47" t="s" s="2">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="P47" t="s" s="2">
         <v>81</v>
@@ -6959,10 +6974,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7071,14 +7086,14 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E49" s="2"/>
       <c r="F49" t="s" s="2">
@@ -7100,13 +7115,13 @@
         <v>134</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="N49" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
@@ -7185,10 +7200,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7214,13 +7229,13 @@
         <v>103</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N50" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
@@ -7228,7 +7243,7 @@
       </c>
       <c r="Q50" s="2"/>
       <c r="R50" t="s" s="2">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="S50" t="s" s="2">
         <v>81</v>
@@ -7270,7 +7285,7 @@
         <v>81</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>89</v>
@@ -7299,10 +7314,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7325,13 +7340,13 @@
         <v>81</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -7382,7 +7397,7 @@
         <v>81</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>79</v>
@@ -7411,13 +7426,13 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C52" t="s" s="2">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D52" t="s" s="2">
         <v>81</v>
@@ -7442,16 +7457,16 @@
         <v>134</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="N52" t="s" s="2">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="O52" t="s" s="2">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="P52" t="s" s="2">
         <v>81</v>
@@ -7529,10 +7544,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7641,14 +7656,14 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E54" s="2"/>
       <c r="F54" t="s" s="2">
@@ -7670,13 +7685,13 @@
         <v>134</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="N54" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="O54" s="2"/>
       <c r="P54" t="s" s="2">
@@ -7755,10 +7770,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -7784,13 +7799,13 @@
         <v>103</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N55" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
@@ -7798,7 +7813,7 @@
       </c>
       <c r="Q55" s="2"/>
       <c r="R55" t="s" s="2">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="S55" t="s" s="2">
         <v>81</v>
@@ -7840,7 +7855,7 @@
         <v>81</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>89</v>
@@ -7869,10 +7884,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -7895,13 +7910,13 @@
         <v>81</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
@@ -7952,7 +7967,7 @@
         <v>81</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>79</v>
@@ -7981,10 +7996,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8010,13 +8025,13 @@
         <v>103</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N57" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
@@ -8024,7 +8039,7 @@
       </c>
       <c r="Q57" s="2"/>
       <c r="R57" t="s" s="2">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="S57" t="s" s="2">
         <v>81</v>
@@ -8066,7 +8081,7 @@
         <v>81</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>89</v>
@@ -8095,10 +8110,10 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8121,13 +8136,13 @@
         <v>81</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -8178,7 +8193,7 @@
         <v>81</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>79</v>
@@ -8207,13 +8222,13 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C59" t="s" s="2">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D59" t="s" s="2">
         <v>81</v>
@@ -8238,16 +8253,16 @@
         <v>134</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="N59" t="s" s="2">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="O59" t="s" s="2">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="P59" t="s" s="2">
         <v>81</v>
@@ -8325,10 +8340,10 @@
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -8437,14 +8452,14 @@
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E61" s="2"/>
       <c r="F61" t="s" s="2">
@@ -8466,13 +8481,13 @@
         <v>134</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="N61" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -8551,10 +8566,10 @@
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -8580,13 +8595,13 @@
         <v>103</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N62" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O62" s="2"/>
       <c r="P62" t="s" s="2">
@@ -8594,7 +8609,7 @@
       </c>
       <c r="Q62" s="2"/>
       <c r="R62" t="s" s="2">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="S62" t="s" s="2">
         <v>81</v>
@@ -8636,7 +8651,7 @@
         <v>81</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>89</v>
@@ -8665,10 +8680,10 @@
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -8691,13 +8706,13 @@
         <v>81</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
@@ -8748,7 +8763,7 @@
         <v>81</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>79</v>
@@ -8777,10 +8792,10 @@
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -8806,13 +8821,13 @@
         <v>103</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N64" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O64" s="2"/>
       <c r="P64" t="s" s="2">
@@ -8820,7 +8835,7 @@
       </c>
       <c r="Q64" s="2"/>
       <c r="R64" t="s" s="2">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="S64" t="s" s="2">
         <v>81</v>
@@ -8862,7 +8877,7 @@
         <v>81</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>89</v>
@@ -8891,10 +8906,10 @@
     </row>
     <row r="65">
       <c r="A65" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -8917,13 +8932,13 @@
         <v>81</v>
       </c>
       <c r="K65" t="s" s="2">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
@@ -8974,7 +8989,7 @@
         <v>81</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>79</v>
@@ -9003,13 +9018,13 @@
     </row>
     <row r="66">
       <c r="A66" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C66" t="s" s="2">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D66" t="s" s="2">
         <v>81</v>
@@ -9034,16 +9049,16 @@
         <v>134</v>
       </c>
       <c r="L66" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="M66" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="N66" t="s" s="2">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="O66" t="s" s="2">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="P66" t="s" s="2">
         <v>81</v>
@@ -9121,10 +9136,10 @@
     </row>
     <row r="67">
       <c r="A67" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -9233,14 +9248,14 @@
     </row>
     <row r="68">
       <c r="A68" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E68" s="2"/>
       <c r="F68" t="s" s="2">
@@ -9262,13 +9277,13 @@
         <v>134</v>
       </c>
       <c r="L68" t="s" s="2">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="N68" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="O68" s="2"/>
       <c r="P68" t="s" s="2">
@@ -9347,10 +9362,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -9376,13 +9391,13 @@
         <v>103</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N69" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
@@ -9390,7 +9405,7 @@
       </c>
       <c r="Q69" s="2"/>
       <c r="R69" t="s" s="2">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="S69" t="s" s="2">
         <v>81</v>
@@ -9432,7 +9447,7 @@
         <v>81</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>89</v>
@@ -9461,10 +9476,10 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -9487,13 +9502,13 @@
         <v>81</v>
       </c>
       <c r="K70" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
@@ -9544,7 +9559,7 @@
         <v>81</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>79</v>
@@ -9573,10 +9588,10 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -9602,13 +9617,13 @@
         <v>103</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N71" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O71" s="2"/>
       <c r="P71" t="s" s="2">
@@ -9616,7 +9631,7 @@
       </c>
       <c r="Q71" s="2"/>
       <c r="R71" t="s" s="2">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="S71" t="s" s="2">
         <v>81</v>
@@ -9658,7 +9673,7 @@
         <v>81</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>89</v>
@@ -9687,10 +9702,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -9713,13 +9728,13 @@
         <v>81</v>
       </c>
       <c r="K72" t="s" s="2">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
@@ -9770,7 +9785,7 @@
         <v>81</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>79</v>
@@ -9799,13 +9814,13 @@
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B73" t="s" s="2">
         <v>156</v>
       </c>
       <c r="C73" t="s" s="2">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="D73" t="s" s="2">
         <v>81</v>
@@ -9830,16 +9845,16 @@
         <v>134</v>
       </c>
       <c r="L73" t="s" s="2">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="M73" t="s" s="2">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="N73" t="s" s="2">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="O73" t="s" s="2">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="P73" t="s" s="2">
         <v>81</v>
@@ -9917,10 +9932,10 @@
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -10029,14 +10044,14 @@
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E75" s="2"/>
       <c r="F75" t="s" s="2">
@@ -10058,13 +10073,13 @@
         <v>134</v>
       </c>
       <c r="L75" t="s" s="2">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="M75" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="N75" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="O75" s="2"/>
       <c r="P75" t="s" s="2">
@@ -10143,10 +10158,10 @@
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -10172,13 +10187,13 @@
         <v>103</v>
       </c>
       <c r="L76" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M76" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N76" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O76" s="2"/>
       <c r="P76" t="s" s="2">
@@ -10186,7 +10201,7 @@
       </c>
       <c r="Q76" s="2"/>
       <c r="R76" t="s" s="2">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="S76" t="s" s="2">
         <v>81</v>
@@ -10228,7 +10243,7 @@
         <v>81</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>89</v>
@@ -10257,10 +10272,10 @@
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -10283,13 +10298,13 @@
         <v>81</v>
       </c>
       <c r="K77" t="s" s="2">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="L77" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="M77" t="s" s="2">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="N77" s="2"/>
       <c r="O77" s="2"/>
@@ -10340,7 +10355,7 @@
         <v>81</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>79</v>
@@ -10369,13 +10384,13 @@
     </row>
     <row r="78">
       <c r="A78" t="s" s="2">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B78" t="s" s="2">
         <v>156</v>
       </c>
       <c r="C78" t="s" s="2">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D78" t="s" s="2">
         <v>81</v>
@@ -10400,7 +10415,7 @@
         <v>134</v>
       </c>
       <c r="L78" t="s" s="2">
-        <v>135</v>
+        <v>327</v>
       </c>
       <c r="M78" t="s" s="2">
         <v>136</v>
@@ -10483,10 +10498,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s" s="2">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -10595,10 +10610,10 @@
     </row>
     <row r="80">
       <c r="A80" t="s" s="2">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -10707,10 +10722,10 @@
     </row>
     <row r="81">
       <c r="A81" t="s" s="2">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -10736,13 +10751,13 @@
         <v>103</v>
       </c>
       <c r="L81" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M81" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N81" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O81" s="2"/>
       <c r="P81" t="s" s="2">
@@ -10750,7 +10765,7 @@
       </c>
       <c r="Q81" s="2"/>
       <c r="R81" t="s" s="2">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="S81" t="s" s="2">
         <v>81</v>
@@ -10792,7 +10807,7 @@
         <v>81</v>
       </c>
       <c r="AF81" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>89</v>
@@ -10821,10 +10836,10 @@
     </row>
     <row r="82">
       <c r="A82" t="s" s="2">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -10847,13 +10862,13 @@
         <v>81</v>
       </c>
       <c r="K82" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L82" t="s" s="2">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="M82" t="s" s="2">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="N82" s="2"/>
       <c r="O82" s="2"/>
@@ -10880,11 +10895,11 @@
         <v>81</v>
       </c>
       <c r="X82" t="s" s="2">
-        <v>113</v>
+        <v>334</v>
       </c>
       <c r="Y82" s="2"/>
       <c r="Z82" t="s" s="2">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="AA82" t="s" s="2">
         <v>81</v>
@@ -10902,7 +10917,7 @@
         <v>81</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>79</v>
@@ -10931,10 +10946,10 @@
     </row>
     <row r="83">
       <c r="A83" t="s" s="2">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -10960,13 +10975,13 @@
         <v>103</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N83" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O83" s="2"/>
       <c r="P83" t="s" s="2">
@@ -10974,7 +10989,7 @@
       </c>
       <c r="Q83" s="2"/>
       <c r="R83" t="s" s="2">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="S83" t="s" s="2">
         <v>81</v>
@@ -11016,7 +11031,7 @@
         <v>81</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>89</v>
@@ -11045,10 +11060,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -11071,13 +11086,13 @@
         <v>81</v>
       </c>
       <c r="K84" t="s" s="2">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="L84" t="s" s="2">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M84" t="s" s="2">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="N84" s="2"/>
       <c r="O84" s="2"/>
@@ -11128,7 +11143,7 @@
         <v>81</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>79</v>
@@ -11157,14 +11172,14 @@
     </row>
     <row r="85">
       <c r="A85" t="s" s="2">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E85" s="2"/>
       <c r="F85" t="s" s="2">
@@ -11186,16 +11201,16 @@
         <v>134</v>
       </c>
       <c r="L85" t="s" s="2">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="M85" t="s" s="2">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="N85" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="O85" t="s" s="2">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="P85" t="s" s="2">
         <v>81</v>
@@ -11244,7 +11259,7 @@
         <v>81</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>79</v>
@@ -11273,10 +11288,10 @@
     </row>
     <row r="86">
       <c r="A86" t="s" s="2">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -11299,13 +11314,13 @@
         <v>90</v>
       </c>
       <c r="K86" t="s" s="2">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="L86" t="s" s="2">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="M86" t="s" s="2">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="N86" s="2"/>
       <c r="O86" s="2"/>
@@ -11356,7 +11371,7 @@
         <v>81</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>79</v>
@@ -11371,13 +11386,13 @@
         <v>101</v>
       </c>
       <c r="AK86" t="s" s="2">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="AL86" t="s" s="2">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="AM86" t="s" s="2">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="AN86" t="s" s="2">
         <v>81</v>
@@ -11385,10 +11400,10 @@
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -11411,70 +11426,70 @@
         <v>90</v>
       </c>
       <c r="K87" t="s" s="2">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="M87" t="s" s="2">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="N87" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="O87" t="s" s="2">
+        <v>358</v>
+      </c>
+      <c r="P87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q87" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="R87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF87" t="s" s="2">
         <v>353</v>
-      </c>
-      <c r="O87" t="s" s="2">
-        <v>354</v>
-      </c>
-      <c r="P87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Q87" t="s" s="2">
-        <v>355</v>
-      </c>
-      <c r="R87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="S87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="T87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="U87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="V87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="W87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="X87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Y87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Z87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AA87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF87" t="s" s="2">
-        <v>349</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>79</v>
@@ -11489,13 +11504,13 @@
         <v>101</v>
       </c>
       <c r="AK87" t="s" s="2">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="AL87" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM87" t="s" s="2">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="AN87" t="s" s="2">
         <v>81</v>
@@ -11503,10 +11518,10 @@
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -11529,16 +11544,16 @@
         <v>90</v>
       </c>
       <c r="K88" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="M88" t="s" s="2">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="N88" t="s" s="2">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="O88" s="2"/>
       <c r="P88" t="s" s="2">
@@ -11568,25 +11583,25 @@
       </c>
       <c r="Y88" s="2"/>
       <c r="Z88" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="AA88" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB88" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC88" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD88" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE88" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF88" t="s" s="2">
         <v>362</v>
-      </c>
-      <c r="AA88" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB88" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC88" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD88" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE88" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF88" t="s" s="2">
-        <v>358</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>79</v>
@@ -11607,18 +11622,18 @@
         <v>81</v>
       </c>
       <c r="AM88" t="s" s="2">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="AN88" t="s" s="2">
-        <v>364</v>
+        <v>368</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s" s="2">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -11641,13 +11656,13 @@
         <v>90</v>
       </c>
       <c r="K89" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L89" t="s" s="2">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="M89" t="s" s="2">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="N89" s="2"/>
       <c r="O89" s="2"/>
@@ -11674,29 +11689,31 @@
         <v>81</v>
       </c>
       <c r="X89" t="s" s="2">
-        <v>368</v>
-      </c>
-      <c r="Y89" s="2"/>
+        <v>372</v>
+      </c>
+      <c r="Y89" t="s" s="2">
+        <v>373</v>
+      </c>
       <c r="Z89" t="s" s="2">
+        <v>374</v>
+      </c>
+      <c r="AA89" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB89" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC89" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD89" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE89" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF89" t="s" s="2">
         <v>369</v>
-      </c>
-      <c r="AA89" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB89" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC89" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD89" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE89" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF89" t="s" s="2">
-        <v>365</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>79</v>
@@ -11711,24 +11728,24 @@
         <v>101</v>
       </c>
       <c r="AK89" t="s" s="2">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="AL89" t="s" s="2">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="AM89" t="s" s="2">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="AN89" t="s" s="2">
-        <v>372</v>
+        <v>377</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s" s="2">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -11751,13 +11768,13 @@
         <v>81</v>
       </c>
       <c r="K90" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L90" t="s" s="2">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="M90" t="s" s="2">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="N90" s="2"/>
       <c r="O90" s="2"/>
@@ -11784,11 +11801,13 @@
         <v>81</v>
       </c>
       <c r="X90" t="s" s="2">
-        <v>376</v>
-      </c>
-      <c r="Y90" s="2"/>
+        <v>372</v>
+      </c>
+      <c r="Y90" t="s" s="2">
+        <v>381</v>
+      </c>
       <c r="Z90" t="s" s="2">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="AA90" t="s" s="2">
         <v>81</v>
@@ -11806,7 +11825,7 @@
         <v>81</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>79</v>
@@ -11821,24 +11840,24 @@
         <v>101</v>
       </c>
       <c r="AK90" t="s" s="2">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="AL90" t="s" s="2">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="AM90" t="s" s="2">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="AN90" t="s" s="2">
-        <v>379</v>
+        <v>384</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s" s="2">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -11864,13 +11883,13 @@
         <v>150</v>
       </c>
       <c r="L91" t="s" s="2">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="M91" t="s" s="2">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="N91" t="s" s="2">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="O91" s="2"/>
       <c r="P91" t="s" s="2">
@@ -11920,7 +11939,7 @@
         <v>81</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>79</v>
@@ -11935,24 +11954,24 @@
         <v>101</v>
       </c>
       <c r="AK91" t="s" s="2">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="AL91" t="s" s="2">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="AM91" t="s" s="2">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="AN91" t="s" s="2">
-        <v>386</v>
+        <v>391</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s" s="2">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -11975,13 +11994,13 @@
         <v>81</v>
       </c>
       <c r="K92" t="s" s="2">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="L92" t="s" s="2">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="M92" t="s" s="2">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="N92" s="2"/>
       <c r="O92" s="2"/>
@@ -12032,7 +12051,7 @@
         <v>81</v>
       </c>
       <c r="AF92" t="s" s="2">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="AG92" t="s" s="2">
         <v>79</v>
@@ -12047,24 +12066,24 @@
         <v>101</v>
       </c>
       <c r="AK92" t="s" s="2">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="AL92" t="s" s="2">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="AM92" t="s" s="2">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="AN92" t="s" s="2">
-        <v>393</v>
+        <v>398</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -12087,13 +12106,13 @@
         <v>90</v>
       </c>
       <c r="K93" t="s" s="2">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="M93" t="s" s="2">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="N93" s="2"/>
       <c r="O93" s="2"/>
@@ -12144,7 +12163,7 @@
         <v>81</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>89</v>
@@ -12159,16 +12178,16 @@
         <v>101</v>
       </c>
       <c r="AK93" t="s" s="2">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="AL93" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM93" t="s" s="2">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="AN93" t="s" s="2">
-        <v>400</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>